<commit_message>
Update the SIT and As and When Commission templates.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Template/As and When Commission.xlsx
+++ b/Template/As and When Commission.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8400"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="11-09-26" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>As And When Commission Daily Status Report</t>
   </si>
@@ -319,7 +319,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="49">
+  <fills count="48">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -461,12 +461,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -820,76 +814,76 @@
     <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -943,7 +937,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1613,7 +1607,9 @@
       </c>
     </row>
     <row r="5" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:9">
-      <c r="B5" s="16"/>
+      <c r="B5" s="16" t="s">
+        <v>7</v>
+      </c>
       <c r="C5" s="17">
         <f t="shared" ref="C5:H5" si="0">SUM(C4:C4)</f>
         <v>0</v>
@@ -1715,7 +1711,7 @@
       <c r="D13" s="36"/>
       <c r="E13" s="36"/>
       <c r="F13" s="37" t="e">
-        <f>(D12+E12)/G12</f>
+        <f>(C12+E12)/G12</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G13" s="37"/>

</xml_diff>